<commit_message>
Mappings -> Match mappings with the changes made to Instalation Profile.
</commit_message>
<xml_diff>
--- a/xlsx/Lists.xlsx
+++ b/xlsx/Lists.xlsx
@@ -1,32 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/o_ugur_exeter_ac_uk/Documents/Desktop/git/metadata-schema/xlsx/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/o_ugur_exeter_ac_uk/Documents/Desktop/rc1.2_ou/metadata-schema/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF7DB5C8-0506-4B86-A706-8965F41E9739}"/>
+  <xr:revisionPtr revIDLastSave="216" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DB7EF3E-118E-4E93-9B61-FB63236E7660}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Languages" sheetId="2" r:id="rId1"/>
     <sheet name="02_Themes" sheetId="3" r:id="rId2"/>
     <sheet name="03_Cultural Context" sheetId="4" r:id="rId3"/>
     <sheet name="04_Social Groups" sheetId="5" r:id="rId4"/>
-    <sheet name="05_Licences" sheetId="6" r:id="rId5"/>
+    <sheet name="05_Rights" sheetId="6" r:id="rId5"/>
     <sheet name="06_Gender" sheetId="7" r:id="rId6"/>
     <sheet name="07_Cultural Sensitivity" sheetId="8" r:id="rId7"/>
     <sheet name="08_Occupations" sheetId="9" r:id="rId8"/>
     <sheet name="09_Project Types" sheetId="10" r:id="rId9"/>
     <sheet name="10_Project Regions" sheetId="11" r:id="rId10"/>
-    <sheet name="11_Rights Statement" sheetId="12" r:id="rId11"/>
-    <sheet name="12_Roles" sheetId="13" r:id="rId12"/>
-    <sheet name="13_Language Labels" sheetId="15" r:id="rId13"/>
-    <sheet name="14_Authority Sources" sheetId="16" r:id="rId14"/>
+    <sheet name="11_Roles" sheetId="13" r:id="rId11"/>
+    <sheet name="12_Language Labels" sheetId="15" r:id="rId12"/>
+    <sheet name="13_Authority Sources" sheetId="16" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="744">
   <si>
     <t>Term ID</t>
   </si>
@@ -1488,60 +1487,24 @@
     <t>Volunteer groups</t>
   </si>
   <si>
-    <t>licence_01</t>
-  </si>
-  <si>
-    <t>CC BY 4.0</t>
-  </si>
-  <si>
     <t>Attribution---This licence lets others distribute, remix, adapt, and build upon your work, even commercially, as long as they credit you for the original creation. This is the most accommodating of licences offered. Recommended for maximum dissemination and use of licenced materials.</t>
   </si>
   <si>
-    <t>licence_02</t>
-  </si>
-  <si>
-    <t>CC BY-SA 4.0</t>
-  </si>
-  <si>
     <t>Attribution-ShareAlike---This licence lets others remix, adapt, and build upon your work even for commercial purposes, as long as they credit you and licence their new creations under the identical terms. This licence is often compared to “copyleft” free and open source software licences. All new works based on yours will carry the same licence, so any derivatives will also allow commercial use. This is the licence used by Wikipedia, and is recommended for materials that would benefit from incorporating content from Wikipedia and similarly licenced projects.</t>
   </si>
   <si>
-    <t>licence_03</t>
-  </si>
-  <si>
-    <t>CC BY-ND 4.0</t>
-  </si>
-  <si>
     <t>Attribution-NoDerivs---This licence lets others reuse the work for any purpose, including commercially; however, it cannot be shared with others in adapted form, and credit must be provided to you.</t>
   </si>
   <si>
-    <t>licence_04</t>
-  </si>
-  <si>
-    <t>CC BY-NC-SA 4.0</t>
-  </si>
-  <si>
     <t>Attribution-NonCommercial-ShareAlike---This licence lets others remix, adapt, and build upon your work non-commercially, as long as they credit you and licence their new creations under the identical terms.</t>
   </si>
   <si>
-    <t>licence_05</t>
-  </si>
-  <si>
-    <t>CC BY-NC-ND 4.0</t>
-  </si>
-  <si>
     <t>Attribution-NonCommercial-NoDerivs---This licence is the most restrictive of our six main licences, only allowing others to download your works and share them with others as long as they credit you, but they can’t change them in any way or use them commercially.</t>
   </si>
   <si>
-    <t>licence_06</t>
-  </si>
-  <si>
     <t>CC0</t>
   </si>
   <si>
-    <t>Public Domain--- is a public dedication tool, which allows creators to give up their copyright and put their works into the worldwide public domain. CC0 allows reusers to distribute, remix, adapt, and build upon the material in any medium or format, with no conditions.</t>
-  </si>
-  <si>
     <t>gender_001</t>
   </si>
   <si>
@@ -2055,108 +2018,72 @@
     <t>North America</t>
   </si>
   <si>
-    <t>rs_001</t>
-  </si>
-  <si>
     <t>In Copyright (InC)</t>
   </si>
   <si>
     <t>indicates that the Item labeled with this Rights Statement is in copyright.</t>
   </si>
   <si>
-    <t>rs_002</t>
-  </si>
-  <si>
     <t>In Copyright - EU Orphan Work (InC-OW-EU)</t>
   </si>
   <si>
     <t>indicates that the Item labeled with this Rights Statement has been identified as an ‘Orphan Work’ under the terms of the EU Orphan Works Directive.</t>
   </si>
   <si>
-    <t>rs_003</t>
-  </si>
-  <si>
     <t>In Copyright - Rights-holder(s) Unlocatable or Unidentifiable (InC-RUU)</t>
   </si>
   <si>
     <t>indicates that the Item labeled with this Rights Statement has been identified as in copyright, but whose rights-holder(s) either cannot be identified or cannot be located.</t>
   </si>
   <si>
-    <t>rs_004</t>
-  </si>
-  <si>
     <t>In Copyright - Educational Use Permitted (InC-EDU)</t>
   </si>
   <si>
     <t>indicates that the Item labeled with this Rights Statement is in copyright but that educational use is allowed without the need to obtain additional permission.</t>
   </si>
   <si>
-    <t>rs_005</t>
-  </si>
-  <si>
     <t>In Copyright - Non-Commercial Use Permitted (InC-NC)</t>
   </si>
   <si>
     <t>indicates that the Item labeled with this Rights Statement is in copyright but that non-commercial use is allowed without the need to obtain additional permission.</t>
   </si>
   <si>
-    <t>rs_006</t>
-  </si>
-  <si>
     <t>No Copyright - Non-Commercial Use Only (NoC-NC)</t>
   </si>
   <si>
     <t>indicates that the underlying Work is in the Public Domain, but the organization that has published the Item is contractually required to allow only non-commercial use by third parties.</t>
   </si>
   <si>
-    <t>rs_007</t>
-  </si>
-  <si>
     <t>No Copyright - Contractual Restrictions (NoC-CR)</t>
   </si>
   <si>
     <t>indicates that the underlying Work is in the Public Domain, but the organization that has published the Item is contractually required to restrict certain forms of use by third parties.</t>
   </si>
   <si>
-    <t>rs_008</t>
-  </si>
-  <si>
     <t>No Copyright - Other Known Legal Restrictions (NoC-OKLR)</t>
   </si>
   <si>
     <t>indicates that the underlying Work is in the Public Domain, but that laws other than copyright impose restrictions on the use of the Item by third parties.</t>
   </si>
   <si>
-    <t>rs_009</t>
-  </si>
-  <si>
     <t>No Copyright - United States (NoC-US)</t>
   </si>
   <si>
     <t>indicates that the underlying Work is in the Public Domain under the laws of the United States, but that a determination was not made as to its copyright status under the copyright laws of other countries.</t>
   </si>
   <si>
-    <t>rs_010</t>
-  </si>
-  <si>
     <t>No Known Copyright (NKC)</t>
   </si>
   <si>
     <t>indicates that the organization that has published the Item believes that no copyright or related rights are known to exist, but that a conclusive determination could not be made.</t>
   </si>
   <si>
-    <t>rs_011</t>
-  </si>
-  <si>
     <t>Copyright Not Evaluated (CNE)</t>
   </si>
   <si>
     <t>indicates that the organization that has published the Item has not evaluated the copyright and related rights status of the Item.</t>
   </si>
   <si>
-    <t>rs_012</t>
-  </si>
-  <si>
     <t>Copyright Undetermined (UND)</t>
   </si>
   <si>
@@ -2263,6 +2190,109 @@
   </si>
   <si>
     <t>MAs Projects</t>
+  </si>
+  <si>
+    <t>Creative Commons - Attribution</t>
+  </si>
+  <si>
+    <t>Creative Commons BY-NC</t>
+  </si>
+  <si>
+    <t>Creative Commons BY-NC-ND</t>
+  </si>
+  <si>
+    <t>Creative Commons BY-NC-SA</t>
+  </si>
+  <si>
+    <t>Creative Commons BY-ND</t>
+  </si>
+  <si>
+    <t>Creative Commons BY-SA</t>
+  </si>
+  <si>
+    <t>Creative Commons 0</t>
+  </si>
+  <si>
+    <t>Public Domain Mark</t>
+  </si>
+  <si>
+    <t>cc_by</t>
+  </si>
+  <si>
+    <t>cc_by_nc</t>
+  </si>
+  <si>
+    <t>cc_by_nc_sa</t>
+  </si>
+  <si>
+    <t>cc_by_nd</t>
+  </si>
+  <si>
+    <t>cc_by_sa</t>
+  </si>
+  <si>
+    <t>inc</t>
+  </si>
+  <si>
+    <t>inc_edu</t>
+  </si>
+  <si>
+    <t>inc_ow_eu</t>
+  </si>
+  <si>
+    <t>inc_nc</t>
+  </si>
+  <si>
+    <t>inc_ruu</t>
+  </si>
+  <si>
+    <t>noc_cr</t>
+  </si>
+  <si>
+    <t>noc_nc</t>
+  </si>
+  <si>
+    <t>noc_oklr</t>
+  </si>
+  <si>
+    <t>noc_us</t>
+  </si>
+  <si>
+    <t>cne</t>
+  </si>
+  <si>
+    <t>und</t>
+  </si>
+  <si>
+    <t>nkc</t>
+  </si>
+  <si>
+    <t>pdm</t>
+  </si>
+  <si>
+    <t>Attribution-NonCommercial 4.0 International---This license enables reusers to distribute, remix, adapt, and build upon the material in any medium or format for noncommercial purposes only, and only so long as attribution is given to the creator.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cc_by_nc_nd </t>
+  </si>
+  <si>
+    <t>CC0 (“CC Zero”) is intended for use only
+by authors or holders of copyright and
+related rights (including database rights), in connection
+with works that are still subject to those rights in one or
+more countries.
+When CC0 is applied to a work, copyright and related
+rights are relinquished worldwide, making the work free
+from those restrictions to the greatest extent possible.</t>
+  </si>
+  <si>
+    <t>The Public Domain Mark (PDM) is used
+to label works that are already free of
+known copyright restrictions. Unlike CC0, PDM doesn’t
+change the copyright status of a work.
+PDM can be used by anyone, and is intended for use
+with works that are already free of known copyright
+restrictions throughout the world.</t>
   </si>
 </sst>
 </file>
@@ -2367,7 +2397,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2378,6 +2408,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4541,50 +4574,50 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>658</v>
+        <v>646</v>
       </c>
       <c r="B3" t="s">
-        <v>659</v>
+        <v>647</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>660</v>
+        <v>648</v>
       </c>
       <c r="B4" t="s">
-        <v>661</v>
+        <v>649</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>662</v>
+        <v>650</v>
       </c>
       <c r="B5" t="s">
-        <v>734</v>
+        <v>710</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="B6" t="s">
-        <v>735</v>
+        <v>711</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="B7" t="s">
-        <v>665</v>
+        <v>653</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>666</v>
+        <v>654</v>
       </c>
       <c r="B8" t="s">
-        <v>667</v>
+        <v>655</v>
       </c>
     </row>
   </sheetData>
@@ -4593,188 +4626,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49F6335E-B01C-4EB6-8502-222DDC2744C7}">
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>668</v>
-      </c>
-      <c r="B3" t="s">
-        <v>669</v>
-      </c>
-      <c r="C3" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>671</v>
-      </c>
-      <c r="B4" t="s">
-        <v>672</v>
-      </c>
-      <c r="C4" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>674</v>
-      </c>
-      <c r="B5" t="s">
-        <v>675</v>
-      </c>
-      <c r="C5" t="s">
-        <v>676</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>677</v>
-      </c>
-      <c r="B6" t="s">
-        <v>678</v>
-      </c>
-      <c r="C6" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>680</v>
-      </c>
-      <c r="B7" t="s">
-        <v>681</v>
-      </c>
-      <c r="C7" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>683</v>
-      </c>
-      <c r="B8" t="s">
-        <v>684</v>
-      </c>
-      <c r="C8" t="s">
-        <v>685</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>686</v>
-      </c>
-      <c r="B9" t="s">
-        <v>687</v>
-      </c>
-      <c r="C9" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>689</v>
-      </c>
-      <c r="B10" t="s">
-        <v>690</v>
-      </c>
-      <c r="C10" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>692</v>
-      </c>
-      <c r="B11" t="s">
-        <v>693</v>
-      </c>
-      <c r="C11" t="s">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>695</v>
-      </c>
-      <c r="B12" t="s">
-        <v>696</v>
-      </c>
-      <c r="C12" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>698</v>
-      </c>
-      <c r="B13" t="s">
-        <v>699</v>
-      </c>
-      <c r="C13" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>701</v>
-      </c>
-      <c r="B14" t="s">
-        <v>702</v>
-      </c>
-      <c r="C14" t="s">
-        <v>703</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F350B9F1-06F7-4E8A-B44A-16E139FB0B1D}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4801,58 +4652,58 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>704</v>
+        <v>680</v>
       </c>
       <c r="B2" t="s">
-        <v>705</v>
+        <v>681</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>706</v>
+        <v>682</v>
       </c>
       <c r="B3" t="s">
-        <v>707</v>
+        <v>683</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>708</v>
+        <v>684</v>
       </c>
       <c r="B4" t="s">
-        <v>709</v>
+        <v>685</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>710</v>
+        <v>686</v>
       </c>
       <c r="B5" t="s">
-        <v>711</v>
+        <v>687</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>712</v>
+        <v>688</v>
       </c>
       <c r="B6" t="s">
-        <v>713</v>
+        <v>689</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>714</v>
+        <v>690</v>
       </c>
       <c r="B7" t="s">
-        <v>715</v>
+        <v>691</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>716</v>
+        <v>692</v>
       </c>
       <c r="B8" t="s">
-        <v>717</v>
+        <v>693</v>
       </c>
     </row>
   </sheetData>
@@ -4860,7 +4711,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5D6CC2-7C88-44F7-8C63-8AD47A42CD2B}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4887,18 +4738,18 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>720</v>
+        <v>696</v>
       </c>
       <c r="B2" t="s">
-        <v>718</v>
+        <v>694</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>721</v>
+        <v>697</v>
       </c>
       <c r="B3" t="s">
-        <v>719</v>
+        <v>695</v>
       </c>
     </row>
   </sheetData>
@@ -4907,7 +4758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9990D756-E521-44BC-87A8-D4E80EBBCAC7}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4934,46 +4785,46 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>724</v>
+        <v>700</v>
       </c>
       <c r="B2" t="s">
-        <v>722</v>
+        <v>698</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>730</v>
+        <v>706</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>725</v>
+        <v>701</v>
       </c>
       <c r="B3" t="s">
-        <v>723</v>
+        <v>699</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>733</v>
+        <v>709</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>726</v>
+        <v>702</v>
       </c>
       <c r="B4" t="s">
-        <v>728</v>
+        <v>704</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>731</v>
+        <v>707</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>727</v>
+        <v>703</v>
       </c>
       <c r="B5" t="s">
-        <v>729</v>
+        <v>705</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>732</v>
+        <v>708</v>
       </c>
     </row>
   </sheetData>
@@ -4986,6 +4837,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{477AB8E0-193B-4ACE-9281-1EB5DE711D3C}">
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
@@ -6022,8 +5877,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B29326D-C093-4910-A1C0-5F486B1575C8}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
+    <col min="2" max="2" width="59.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="100.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
@@ -6067,69 +5927,235 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>722</v>
+      </c>
+      <c r="B3" t="s">
+        <v>714</v>
+      </c>
+      <c r="C3" t="s">
         <v>479</v>
-      </c>
-      <c r="B3" t="s">
-        <v>480</v>
-      </c>
-      <c r="C3" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>482</v>
+        <v>723</v>
       </c>
       <c r="B4" t="s">
-        <v>483</v>
+        <v>715</v>
       </c>
       <c r="C4" t="s">
-        <v>484</v>
+        <v>740</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>485</v>
+        <v>741</v>
       </c>
       <c r="B5" t="s">
-        <v>486</v>
+        <v>716</v>
       </c>
       <c r="C5" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>488</v>
+        <v>724</v>
       </c>
       <c r="B6" t="s">
-        <v>489</v>
+        <v>717</v>
       </c>
       <c r="C6" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>491</v>
+        <v>725</v>
       </c>
       <c r="B7" t="s">
-        <v>492</v>
+        <v>718</v>
       </c>
       <c r="C7" t="s">
-        <v>493</v>
+        <v>481</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>494</v>
+        <v>726</v>
       </c>
       <c r="B8" t="s">
-        <v>495</v>
+        <v>719</v>
       </c>
       <c r="C8" t="s">
-        <v>496</v>
-      </c>
+        <v>480</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>727</v>
+      </c>
+      <c r="B9" t="s">
+        <v>656</v>
+      </c>
+      <c r="C9" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>728</v>
+      </c>
+      <c r="B10" t="s">
+        <v>662</v>
+      </c>
+      <c r="C10" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>729</v>
+      </c>
+      <c r="B11" t="s">
+        <v>658</v>
+      </c>
+      <c r="C11" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>730</v>
+      </c>
+      <c r="B12" t="s">
+        <v>664</v>
+      </c>
+      <c r="C12" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>731</v>
+      </c>
+      <c r="B13" t="s">
+        <v>660</v>
+      </c>
+      <c r="C13" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>732</v>
+      </c>
+      <c r="B14" t="s">
+        <v>668</v>
+      </c>
+      <c r="C14" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>733</v>
+      </c>
+      <c r="B15" t="s">
+        <v>666</v>
+      </c>
+      <c r="C15" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>734</v>
+      </c>
+      <c r="B16" t="s">
+        <v>670</v>
+      </c>
+      <c r="C16" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>735</v>
+      </c>
+      <c r="B17" t="s">
+        <v>672</v>
+      </c>
+      <c r="C17" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>736</v>
+      </c>
+      <c r="B18" t="s">
+        <v>676</v>
+      </c>
+      <c r="C18" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>737</v>
+      </c>
+      <c r="B19" t="s">
+        <v>678</v>
+      </c>
+      <c r="C19" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>738</v>
+      </c>
+      <c r="B20" t="s">
+        <v>674</v>
+      </c>
+      <c r="C20" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>484</v>
+      </c>
+      <c r="B21" t="s">
+        <v>720</v>
+      </c>
+      <c r="C21" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>739</v>
+      </c>
+      <c r="B22" t="s">
+        <v>721</v>
+      </c>
+      <c r="C22" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C23" s="9"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C24" s="9"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C25" s="9"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C26" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6183,35 +6209,35 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>497</v>
+        <v>485</v>
       </c>
       <c r="B3" t="s">
-        <v>498</v>
+        <v>486</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>499</v>
+        <v>487</v>
       </c>
       <c r="B4" t="s">
-        <v>500</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>501</v>
+        <v>489</v>
       </c>
       <c r="B5" t="s">
-        <v>502</v>
+        <v>490</v>
       </c>
       <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>503</v>
+        <v>491</v>
       </c>
       <c r="B6" t="s">
-        <v>504</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -6269,35 +6295,35 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>505</v>
+        <v>493</v>
       </c>
       <c r="B3" t="s">
-        <v>506</v>
+        <v>494</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>507</v>
+        <v>495</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>508</v>
+        <v>496</v>
       </c>
       <c r="B4" t="s">
-        <v>509</v>
+        <v>497</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>510</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>511</v>
+        <v>499</v>
       </c>
       <c r="B5" t="s">
-        <v>512</v>
+        <v>500</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>513</v>
+        <v>501</v>
       </c>
     </row>
   </sheetData>
@@ -6354,549 +6380,549 @@
         <v>5</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>514</v>
+        <v>502</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>515</v>
+        <v>503</v>
       </c>
       <c r="B3" t="s">
-        <v>516</v>
+        <v>504</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>517</v>
+        <v>505</v>
       </c>
       <c r="B4" t="s">
-        <v>518</v>
+        <v>506</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>519</v>
+        <v>507</v>
       </c>
       <c r="B5" t="s">
-        <v>520</v>
+        <v>508</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>521</v>
+        <v>509</v>
       </c>
       <c r="B6" t="s">
-        <v>522</v>
+        <v>510</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="B7" t="s">
-        <v>524</v>
+        <v>512</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>525</v>
+        <v>513</v>
       </c>
       <c r="B8" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>527</v>
+        <v>515</v>
       </c>
       <c r="B9" t="s">
-        <v>528</v>
+        <v>516</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>529</v>
+        <v>517</v>
       </c>
       <c r="B10" t="s">
-        <v>530</v>
+        <v>518</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>531</v>
+        <v>519</v>
       </c>
       <c r="B11" t="s">
-        <v>532</v>
+        <v>520</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>533</v>
+        <v>521</v>
       </c>
       <c r="B12" t="s">
-        <v>534</v>
+        <v>522</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>535</v>
+        <v>523</v>
       </c>
       <c r="B13" t="s">
-        <v>536</v>
+        <v>524</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>537</v>
+        <v>525</v>
       </c>
       <c r="B14" t="s">
-        <v>538</v>
+        <v>526</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>539</v>
+        <v>527</v>
       </c>
       <c r="B15" t="s">
-        <v>540</v>
+        <v>528</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>541</v>
+        <v>529</v>
       </c>
       <c r="B16" t="s">
-        <v>542</v>
+        <v>530</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>543</v>
+        <v>531</v>
       </c>
       <c r="B17" t="s">
-        <v>544</v>
+        <v>532</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>545</v>
+        <v>533</v>
       </c>
       <c r="B18" t="s">
-        <v>546</v>
+        <v>534</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>547</v>
+        <v>535</v>
       </c>
       <c r="B19" t="s">
-        <v>548</v>
+        <v>536</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>549</v>
+        <v>537</v>
       </c>
       <c r="B20" t="s">
-        <v>550</v>
+        <v>538</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>551</v>
+        <v>539</v>
       </c>
       <c r="B21" t="s">
-        <v>552</v>
+        <v>540</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>553</v>
+        <v>541</v>
       </c>
       <c r="B22" t="s">
-        <v>554</v>
+        <v>542</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>555</v>
+        <v>543</v>
       </c>
       <c r="B23" t="s">
-        <v>556</v>
+        <v>544</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>557</v>
+        <v>545</v>
       </c>
       <c r="B24" t="s">
-        <v>558</v>
+        <v>546</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>559</v>
+        <v>547</v>
       </c>
       <c r="B25" t="s">
-        <v>560</v>
+        <v>548</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>561</v>
+        <v>549</v>
       </c>
       <c r="B26" t="s">
-        <v>562</v>
+        <v>550</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>563</v>
+        <v>551</v>
       </c>
       <c r="B27" t="s">
-        <v>564</v>
+        <v>552</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>565</v>
+        <v>553</v>
       </c>
       <c r="B28" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>567</v>
+        <v>555</v>
       </c>
       <c r="B29" t="s">
-        <v>568</v>
+        <v>556</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>569</v>
+        <v>557</v>
       </c>
       <c r="B30" t="s">
-        <v>570</v>
+        <v>558</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>571</v>
+        <v>559</v>
       </c>
       <c r="B31" t="s">
-        <v>572</v>
+        <v>560</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>573</v>
+        <v>561</v>
       </c>
       <c r="B32" t="s">
-        <v>574</v>
+        <v>562</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>575</v>
+        <v>563</v>
       </c>
       <c r="B33" t="s">
-        <v>576</v>
+        <v>564</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>577</v>
+        <v>565</v>
       </c>
       <c r="B34" t="s">
-        <v>578</v>
+        <v>566</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>579</v>
+        <v>567</v>
       </c>
       <c r="B35" t="s">
-        <v>580</v>
+        <v>568</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>581</v>
+        <v>569</v>
       </c>
       <c r="B36" t="s">
-        <v>582</v>
+        <v>570</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>583</v>
+        <v>571</v>
       </c>
       <c r="B37" t="s">
-        <v>584</v>
+        <v>572</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>585</v>
+        <v>573</v>
       </c>
       <c r="B38" t="s">
-        <v>586</v>
+        <v>574</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>587</v>
+        <v>575</v>
       </c>
       <c r="B39" t="s">
-        <v>588</v>
+        <v>576</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>589</v>
+        <v>577</v>
       </c>
       <c r="B40" t="s">
-        <v>590</v>
+        <v>578</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>591</v>
+        <v>579</v>
       </c>
       <c r="B41" t="s">
-        <v>592</v>
+        <v>580</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>593</v>
+        <v>581</v>
       </c>
       <c r="B42" t="s">
-        <v>594</v>
+        <v>582</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>595</v>
+        <v>583</v>
       </c>
       <c r="B43" t="s">
-        <v>596</v>
+        <v>584</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>597</v>
+        <v>585</v>
       </c>
       <c r="B44" t="s">
-        <v>598</v>
+        <v>586</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>599</v>
+        <v>587</v>
       </c>
       <c r="B45" t="s">
-        <v>600</v>
+        <v>588</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>601</v>
+        <v>589</v>
       </c>
       <c r="B46" t="s">
-        <v>602</v>
+        <v>590</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>603</v>
+        <v>591</v>
       </c>
       <c r="B47" t="s">
-        <v>604</v>
+        <v>592</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>605</v>
+        <v>593</v>
       </c>
       <c r="B48" t="s">
-        <v>606</v>
+        <v>594</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>607</v>
+        <v>595</v>
       </c>
       <c r="B49" t="s">
-        <v>608</v>
+        <v>596</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>609</v>
+        <v>597</v>
       </c>
       <c r="B50" t="s">
-        <v>610</v>
+        <v>598</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>611</v>
+        <v>599</v>
       </c>
       <c r="B51" t="s">
-        <v>612</v>
+        <v>600</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>613</v>
+        <v>601</v>
       </c>
       <c r="B52" t="s">
-        <v>614</v>
+        <v>602</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>615</v>
+        <v>603</v>
       </c>
       <c r="B53" t="s">
-        <v>616</v>
+        <v>604</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="B54" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="B55" t="s">
-        <v>620</v>
+        <v>608</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>621</v>
+        <v>609</v>
       </c>
       <c r="B56" t="s">
-        <v>622</v>
+        <v>610</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>623</v>
+        <v>611</v>
       </c>
       <c r="B57" t="s">
-        <v>624</v>
+        <v>612</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>625</v>
+        <v>613</v>
       </c>
       <c r="B58" t="s">
-        <v>626</v>
+        <v>614</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>627</v>
+        <v>615</v>
       </c>
       <c r="B59" t="s">
-        <v>628</v>
+        <v>616</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>629</v>
+        <v>617</v>
       </c>
       <c r="B60" t="s">
-        <v>630</v>
+        <v>618</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>631</v>
+        <v>619</v>
       </c>
       <c r="B61" t="s">
-        <v>632</v>
+        <v>620</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>633</v>
+        <v>621</v>
       </c>
       <c r="B62" t="s">
-        <v>634</v>
+        <v>622</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>635</v>
+        <v>623</v>
       </c>
       <c r="B63" t="s">
-        <v>636</v>
+        <v>624</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>637</v>
+        <v>625</v>
       </c>
       <c r="B64" t="s">
-        <v>638</v>
+        <v>626</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>639</v>
+        <v>627</v>
       </c>
       <c r="B65" t="s">
-        <v>640</v>
+        <v>628</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>641</v>
+        <v>629</v>
       </c>
       <c r="B66" t="s">
-        <v>642</v>
+        <v>630</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>643</v>
+        <v>631</v>
       </c>
       <c r="B67" t="s">
-        <v>644</v>
+        <v>632</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>645</v>
+        <v>633</v>
       </c>
       <c r="B68" t="s">
-        <v>646</v>
+        <v>634</v>
       </c>
       <c r="C68" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>648</v>
+        <v>636</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>649</v>
+        <v>637</v>
       </c>
       <c r="C69" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
     </row>
   </sheetData>
@@ -6954,42 +6980,42 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>650</v>
+        <v>638</v>
       </c>
       <c r="B3" t="s">
-        <v>651</v>
+        <v>639</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>652</v>
+        <v>640</v>
       </c>
       <c r="B4" t="s">
-        <v>653</v>
+        <v>641</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>654</v>
+        <v>642</v>
       </c>
       <c r="B5" t="s">
-        <v>655</v>
+        <v>643</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>656</v>
+        <v>644</v>
       </c>
       <c r="B6" t="s">
-        <v>657</v>
+        <v>645</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>736</v>
+        <v>712</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>737</v>
+        <v>713</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
traditional knowledge and biocultural labels
</commit_message>
<xml_diff>
--- a/xlsx/Lists.xlsx
+++ b/xlsx/Lists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/o_ugur_exeter_ac_uk/Documents/Desktop/rc1.2_ou/metadata-schema/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="216" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DB7EF3E-118E-4E93-9B61-FB63236E7660}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{168892A6-3CCB-41DC-9029-19331CF7CDF7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1875" yWindow="900" windowWidth="11220" windowHeight="16605" firstSheet="14" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Languages" sheetId="2" r:id="rId1"/>
@@ -26,6 +26,8 @@
     <sheet name="11_Roles" sheetId="13" r:id="rId11"/>
     <sheet name="12_Language Labels" sheetId="15" r:id="rId12"/>
     <sheet name="13_Authority Sources" sheetId="16" r:id="rId13"/>
+    <sheet name="14_Traditional Knowledge Labels" sheetId="17" r:id="rId14"/>
+    <sheet name="15_Biocultural Labels" sheetId="18" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="865">
   <si>
     <t>Term ID</t>
   </si>
@@ -2294,12 +2296,377 @@
 with works that are already free of known copyright
 restrictions throughout the world.</t>
   </si>
+  <si>
+    <t>TK Attribution (TK A)</t>
+  </si>
+  <si>
+    <t>This Label is being used to correct historical mistakes or exclusions pertaining to this material. This is especially in relation to the names of the people involved in performing or making this work and/or correctly naming the community from which it originally derives. As a user you are being asked to also apply the correct attribution in any future use of this work.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-attribution/</t>
+  </si>
+  <si>
+    <t>TK Clan (TK CL)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material is traditionally and usually not publicly available. The Label lets future users know that this material has specific conditions for use and sharing because of clan membership and/or relationships. This material is not, and never was, free, public, or available for everyone. This Label asks viewers of these materials to respect the cultural values and expectations about circulation and use defined by designated clans, members, and their internal relations.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-clan/</t>
+  </si>
+  <si>
+    <t>TK Family (TK F)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material is traditionally and usually not publicly available. The Label is correcting a misunderstanding about the circulation options for this material and letting any users know that this material has specific conditions for sharing between family members. Who these family members are, and how sharing occurs will be defined in each locale. This material is not, and never was, free, public, or available for everyone at anytime. This Label asks you to think about how you are going to use this material and to respect different cultural values and expectations about circulation and use.</t>
+  </si>
+  <si>
+    <t>TK Multiple Communities (TK MC)</t>
+  </si>
+  <si>
+    <t>Responsibility and ownership over this material is spread across several distinct communities. Use will be dependent upon discussion and negotiation with the multiple communities named herein [insert names]. Decisions about use will need to be decided collectively. As an external user of this material you are asked to recognize and respect cultural protocols in relation to the use of this material and clear your intended use with the relevant communities.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-multiple-communities/</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-family/</t>
+  </si>
+  <si>
+    <t>TK Community Voice (TK CV)</t>
+  </si>
+  <si>
+    <t>This Label is being used to encourage the sharing of stories and voices about this material. The Label indicates that existing knowledge or descriptions are incomplete or partial. Any community member is invited and welcome to contribute to our community knowledge about this event, photograph, recording or heritage item. Sharing our voices helps us reclaim our histories and knowledge. This sharing is an internal process.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-community-voice/</t>
+  </si>
+  <si>
+    <t>TK Creative (TK CR)</t>
+  </si>
+  <si>
+    <t>This Label is being used to acknowledge the relationship between the creative practices of [name] and [community name] and the associated cultural responsibilities.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-creative/</t>
+  </si>
+  <si>
+    <t>TK Verified (TK V)</t>
+  </si>
+  <si>
+    <t>This Label affirms that the representation and presentation of this material is in keeping with community expectations and cultural protocols. It lets you know that for the individual, family or community represented in this material, use is considered fair, reasonable and respectful.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-verified/</t>
+  </si>
+  <si>
+    <t>TK Non-Verified (TK NV)</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-non-verified/</t>
+  </si>
+  <si>
+    <t>This Label is being used because there are concerns about accuracy and/or representations made in this material. This material was not created through informed consent or community protocols for research and engagement. Therefore, questions about its accuracy and who/how it represents this community are being raised.</t>
+  </si>
+  <si>
+    <t>TK Seasonal (TK S)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material traditionally and usually is heard and/or utilized at a particular time of year and in response to specific seasonal changes and conditions. For instance, many important ceremonies are held at very specific times of the year. This Label is being used to indicate sophisticated relationships between land and knowledge creation. It is also being used to highlight the relationships between recorded material and the specific contexts where it derives, especially the interconnected and embodied teachings that it conveys.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-seasonal/</t>
+  </si>
+  <si>
+    <t>This material has specific gender restrictions on access. It is usually only to be accessed and used by women in the community. If you are not from the community and you have accessed this material, you are requested not to download, copy, remix or otherwise circulate this material to others without permission. This Label asks you to think about whether you should be using this material and to respect different cultural values and expectations about circulation and use.</t>
+  </si>
+  <si>
+    <t>TK Women General (TK WG)</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-women-general/</t>
+  </si>
+  <si>
+    <t>TK Men General (TK MG)</t>
+  </si>
+  <si>
+    <t>This material has specific gender restrictions on access. It is usually only to be accessed and used by men in the community. If you are not from the community and you have accessed this material, you are requested to not download, copy, remix or otherwise circulate this material to others without permission. This Label asks you to think about whether you should be using this material and to respect different cultural values and expectations about circulation and use.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-men-general/</t>
+  </si>
+  <si>
+    <t>TK Men Restricted (TK MR)</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-men-restricted/</t>
+  </si>
+  <si>
+    <t>This material has specific gender restrictions on access. It is regarded as important secret and/or ceremonial material that has community-based laws in relation to who can access it. Given its nature it is only to be accessed and used by authorized [and/or initiated] men in the community. If you are an external third party user and you have accessed this material, you are requested to not download, copy, remix or otherwise circulate this material to others. This material is not freely available within the community and it therefore should not be considered freely available outside of the community. This Label asks you to think about whether you should be using this material and to respect different cultural values and expectations about circulation and use.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-women-restricted/</t>
+  </si>
+  <si>
+    <t>TK Women Restricted (TK WR)</t>
+  </si>
+  <si>
+    <t>This material has specific gender restrictions on access. It is regarded as important secret and/or ceremonial material that has community-based laws in relation to who can access it. Given its nature it is only to be accessed and used by authorized [and/or initiated] women in the community. If you are an external third party user and you have accessed this material, you are requested to not download, copy, remix or otherwise circulate this material to others. This material is not freely available within the community and it therefore should not be considered freely available outside of the community. This Label asks you to think about whether you should be using this material and to respect different cultural values and expectations about circulation and use.</t>
+  </si>
+  <si>
+    <t>TK Culturally Sensitive (TK CS)</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-culturally-sensitive/</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material has cultural and/or historical sensitivities. The Label asks for care to be taken when this material is accessed, used, and circulated, especially when materials are first returned or reunited with communities of origin. In some instances, this Label will indicate that there are specific permissions for use of this material required directly from the community itself.</t>
+  </si>
+  <si>
+    <t>TK Secret / Sacred (TK SS)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material is traditionally and usually not publicly available because it contains important secret or sacred components. The Label is correcting a misunderstanding about the significance of this material and therefore its circulation conditions. It is letting users know that because of its secret/sacred status it is not, and was never free, public, or available for everyone at anytime. This Label asks you to think about whether you should be using this material and to respect different cultural values and expectations about circulation and use.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-secret-sacred/</t>
+  </si>
+  <si>
+    <t>TK Open to Commercialization (TK OC)</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-commercial/</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that [community name or authorized party] is open to commercialization opportunities that might derive from any cultural material with traditional knowledge to which this Label is connected to. As a primary party for any partnership and collaboration opportunities that emerge from the use of this cultural material and traditional knowledge, we retain an expressed interest in any future negotiations.</t>
+  </si>
+  <si>
+    <t>TK Non-Commercial (TK NC)</t>
+  </si>
+  <si>
+    <t>This material has been designated as being available for non-commercial use. You are allowed to use this material for non-commercial purposes including for research, study, or public presentation and/or online in blogs or non-commercial websites. This Label asks you to think and act with fairness and responsibility towards this material and the original custodians.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-non-commercial/</t>
+  </si>
+  <si>
+    <t>TK Community Use Only (TK CO)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material is traditionally and usually not publicly available. The Label is correcting a misunderstanding about the circulation options for this material and letting any users know that this material has specific conditions for circulation within the community. It is not, and never was, free, public, or available for everyone at anytime. This Label asks you to think about how you are going to use this material and to respect different cultural values and expectations about circulation and use.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-community-use-only/</t>
+  </si>
+  <si>
+    <t>TK Outreach (TK O)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material is traditionally and usually not publicly available. The Label is correcting a misunderstanding about the circulation options for this material and letting any users know that this material can be used for educational outreach activities. This Label asks you to respect the designated circulation conditions for this material and additionally, where possible, to develop a means for fair and equitable reciprocal exchange for the use of this material with the relevant TK holders. This exchange might include access to educational or other resources that are difficult to access under normal circumstances.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-outreach/</t>
+  </si>
+  <si>
+    <t>TK Open to Collaboration (TK CB)</t>
+  </si>
+  <si>
+    <t>This Label is being used to make clear [community name or authorizing body] is open to future engagement, collaboration, and partnership around research opportunities.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/tk-open-to-collaboration/</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>tka</t>
+  </si>
+  <si>
+    <t>tkcl</t>
+  </si>
+  <si>
+    <t>tkf</t>
+  </si>
+  <si>
+    <t>tkmc</t>
+  </si>
+  <si>
+    <t>tkcv</t>
+  </si>
+  <si>
+    <t>tkcr</t>
+  </si>
+  <si>
+    <t>tkv</t>
+  </si>
+  <si>
+    <t>tknv</t>
+  </si>
+  <si>
+    <t>tks</t>
+  </si>
+  <si>
+    <t>tkwg</t>
+  </si>
+  <si>
+    <t>tkmg</t>
+  </si>
+  <si>
+    <t>tkmr</t>
+  </si>
+  <si>
+    <t>tkwr</t>
+  </si>
+  <si>
+    <t>tkcs</t>
+  </si>
+  <si>
+    <t>tkss</t>
+  </si>
+  <si>
+    <t>tkoc</t>
+  </si>
+  <si>
+    <t>tknc</t>
+  </si>
+  <si>
+    <t>tkco</t>
+  </si>
+  <si>
+    <t>tko</t>
+  </si>
+  <si>
+    <t>tkcb</t>
+  </si>
+  <si>
+    <t>BC Provenance (BC P)</t>
+  </si>
+  <si>
+    <t>This Label is being used to affirm an inherent interest Indigenous people have in the scientific collections and data about communities, peoples, and the biodiversity found within traditional lands, waters and territories. [Community name or authorizing party] retains the right to be named and associated with it into the future. This association reflects a significant relationship and responsibility to [the species or biological entity] and associated scientific collections and data.
+[Optional attribution statement]</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-provenance/</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-multiple-communities/</t>
+  </si>
+  <si>
+    <t>BC Multiple Communities (BC MC)</t>
+  </si>
+  <si>
+    <t>This Label is being used to affirm that responsibility and ownership over this information, collection, data, and digital sequence information (DSI) is spread across several distinct communities. Use will be dependent upon discussion and negotiation with these multiple communities.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-clan/</t>
+  </si>
+  <si>
+    <t>BC Clan (BC CL)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that this material is traditionally and usually not publicly available. The Label lets future users know that this data has specific conditions for use and sharing because of clan membership and/or relationships. This Label asks viewers of this data to respect the cultural values and expectations about circulation and use defined by designated clans, members, and their internal relations.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-consent-verified/</t>
+  </si>
+  <si>
+    <t>BC Consent Verified (BC CV)</t>
+  </si>
+  <si>
+    <t>This Label is being used to verify that [community name or authorizing party] have consent conditions in place for the use of this information, collections, data, and digital sequence information. [These can be found at ….].</t>
+  </si>
+  <si>
+    <t>BC Consent Non-Verified (BC CNV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This Label is being used because there are concerns about the accuracy of the consent and/or representations made for this data. This material was not created through informed consent or community protocols for research and engagement. </t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-consent-non-verified/</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-research-use/</t>
+  </si>
+  <si>
+    <t>This Label is being used by [community name or authorizing body] to allow this information, collection, data, and digital sequence information (DSI) to be used for unspecified research purposes. This Label does not provide permission for commercialization activities.
+[Optional return of research results statement]</t>
+  </si>
+  <si>
+    <t>BC Research Use (BC R)</t>
+  </si>
+  <si>
+    <t>This Label is being used to make clear [community name or authorizing body] is open to future engagement, collaboration, and partnership around research and outreach opportunities.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-open-to-collaboration/</t>
+  </si>
+  <si>
+    <t>BC Open to Collaboration (BC CB)</t>
+  </si>
+  <si>
+    <t>BC Open to Commercialization (BC OC)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that [community name or authorizing party] is open to commercialization opportunities that might derive from any information, collections, data, and digital sequence information (DSI) to which this Label is connected. As a primary party in any partnership and collaboration opportunity that emerges from the use of these resources, we retain an express interest in any future negotiations.</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-open-to-commercialization/</t>
+  </si>
+  <si>
+    <t>BC Outreach (BC O)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Label is letting any users know that this data can be used for educational outreach activities. This Label asks you to respect the designated circulation conditions for these biocultural materials and/or data and additionally, where possible, to develop a means for fair and equitable reciprocal exchange for the use of this data with the relevant BC holders. </t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-outreach/</t>
+  </si>
+  <si>
+    <t>https://localcontexts.org/label/bc-non-commercial/</t>
+  </si>
+  <si>
+    <t>BC Non-Commercial (BC NC)</t>
+  </si>
+  <si>
+    <t>This Label is being used to indicate that these biocultural materials and/or data have been designated as being available for non-commercial use. You are allowed to use this material for non-commercial purposes including for research, study, or public presentation and/or online in blogs or non-commercial websites. This Label asks you to think and act with respect and responsibility towards this data and the original custodians.</t>
+  </si>
+  <si>
+    <t>bcp</t>
+  </si>
+  <si>
+    <t>bcmc</t>
+  </si>
+  <si>
+    <t>bccl</t>
+  </si>
+  <si>
+    <t>bccv</t>
+  </si>
+  <si>
+    <t>bccnv</t>
+  </si>
+  <si>
+    <t>bcr</t>
+  </si>
+  <si>
+    <t>bccb</t>
+  </si>
+  <si>
+    <t>bcoc</t>
+  </si>
+  <si>
+    <t>bco</t>
+  </si>
+  <si>
+    <t>bcnc</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2364,6 +2731,12 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF44474A"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2397,7 +2770,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2412,6 +2785,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{7D5AF2CA-6FAC-4DED-9EC5-A1BA931E1331}"/>
@@ -4833,6 +5212,540 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13F67E00-EC1B-4E47-80B8-6C2ADC61550B}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>805</v>
+      </c>
+      <c r="B3" t="s">
+        <v>744</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>745</v>
+      </c>
+      <c r="F3" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>806</v>
+      </c>
+      <c r="B4" t="s">
+        <v>747</v>
+      </c>
+      <c r="C4" t="s">
+        <v>748</v>
+      </c>
+      <c r="F4" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>807</v>
+      </c>
+      <c r="B5" t="s">
+        <v>750</v>
+      </c>
+      <c r="C5" t="s">
+        <v>751</v>
+      </c>
+      <c r="F5" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>808</v>
+      </c>
+      <c r="B6" t="s">
+        <v>752</v>
+      </c>
+      <c r="C6" t="s">
+        <v>753</v>
+      </c>
+      <c r="F6" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>809</v>
+      </c>
+      <c r="B7" t="s">
+        <v>756</v>
+      </c>
+      <c r="C7" t="s">
+        <v>757</v>
+      </c>
+      <c r="F7" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>810</v>
+      </c>
+      <c r="B8" t="s">
+        <v>759</v>
+      </c>
+      <c r="C8" t="s">
+        <v>760</v>
+      </c>
+      <c r="F8" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>811</v>
+      </c>
+      <c r="B9" t="s">
+        <v>762</v>
+      </c>
+      <c r="C9" t="s">
+        <v>763</v>
+      </c>
+      <c r="F9" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>812</v>
+      </c>
+      <c r="B10" t="s">
+        <v>765</v>
+      </c>
+      <c r="C10" t="s">
+        <v>767</v>
+      </c>
+      <c r="F10" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>813</v>
+      </c>
+      <c r="B11" t="s">
+        <v>768</v>
+      </c>
+      <c r="C11" t="s">
+        <v>769</v>
+      </c>
+      <c r="F11" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>814</v>
+      </c>
+      <c r="B12" t="s">
+        <v>772</v>
+      </c>
+      <c r="C12" t="s">
+        <v>771</v>
+      </c>
+      <c r="F12" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>815</v>
+      </c>
+      <c r="B13" t="s">
+        <v>774</v>
+      </c>
+      <c r="C13" t="s">
+        <v>775</v>
+      </c>
+      <c r="F13" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>816</v>
+      </c>
+      <c r="B14" t="s">
+        <v>777</v>
+      </c>
+      <c r="C14" t="s">
+        <v>779</v>
+      </c>
+      <c r="F14" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>817</v>
+      </c>
+      <c r="B15" t="s">
+        <v>781</v>
+      </c>
+      <c r="C15" t="s">
+        <v>782</v>
+      </c>
+      <c r="F15" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>818</v>
+      </c>
+      <c r="B16" t="s">
+        <v>783</v>
+      </c>
+      <c r="C16" t="s">
+        <v>785</v>
+      </c>
+      <c r="F16" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>819</v>
+      </c>
+      <c r="B17" t="s">
+        <v>786</v>
+      </c>
+      <c r="C17" t="s">
+        <v>787</v>
+      </c>
+      <c r="F17" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>820</v>
+      </c>
+      <c r="B18" t="s">
+        <v>789</v>
+      </c>
+      <c r="C18" t="s">
+        <v>791</v>
+      </c>
+      <c r="F18" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>821</v>
+      </c>
+      <c r="B19" t="s">
+        <v>792</v>
+      </c>
+      <c r="C19" t="s">
+        <v>793</v>
+      </c>
+      <c r="F19" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>822</v>
+      </c>
+      <c r="B20" t="s">
+        <v>795</v>
+      </c>
+      <c r="C20" t="s">
+        <v>796</v>
+      </c>
+      <c r="F20" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>823</v>
+      </c>
+      <c r="B21" t="s">
+        <v>798</v>
+      </c>
+      <c r="C21" t="s">
+        <v>799</v>
+      </c>
+      <c r="F21" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>824</v>
+      </c>
+      <c r="B22" t="s">
+        <v>801</v>
+      </c>
+      <c r="C22" t="s">
+        <v>802</v>
+      </c>
+      <c r="F22" t="s">
+        <v>803</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F3B1DC4-7228-4E7B-AE10-2426AE58FF55}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.21875" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.88671875" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.88671875" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="13">
+        <v>1</v>
+      </c>
+      <c r="B1" s="13">
+        <v>2</v>
+      </c>
+      <c r="C1" s="13">
+        <v>3</v>
+      </c>
+      <c r="D1" s="13">
+        <v>4</v>
+      </c>
+      <c r="E1" s="13">
+        <v>5</v>
+      </c>
+      <c r="F1" s="13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
+        <v>855</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>825</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>826</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>856</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>829</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>830</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>857</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>832</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>833</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>858</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>835</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>836</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="12" t="s">
+        <v>859</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>837</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>838</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>860</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>842</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>841</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>861</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>845</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>843</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="12" t="s">
+        <v>862</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>846</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>847</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="12" t="s">
+        <v>863</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>849</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>850</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>864</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>853</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>854</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>852</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F3" r:id="rId1" xr:uid="{1F779799-C8B2-499C-B7ED-E33915A311AB}"/>
+    <hyperlink ref="F12" r:id="rId2" xr:uid="{C28B5BEF-4771-4915-BA25-24C55EFF2E13}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{477AB8E0-193B-4ACE-9281-1EB5DE711D3C}">
   <dimension ref="A1:F32"/>

</xml_diff>

<commit_message>
saved changes before merge
</commit_message>
<xml_diff>
--- a/xlsx/Lists.xlsx
+++ b/xlsx/Lists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/o_ugur_exeter_ac_uk/Documents/Desktop/rc1.2_ou/metadata-schema/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="404" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A227B620-8B34-4065-B621-0B50314FD73C}"/>
+  <xr:revisionPtr revIDLastSave="405" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88ED991A-AE5C-4BF0-A97E-FF7025AB0314}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="18840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="18840" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Languages" sheetId="2" r:id="rId1"/>
@@ -1999,9 +1999,6 @@
     <t>reg_02</t>
   </si>
   <si>
-    <t>Asia Pasific</t>
-  </si>
-  <si>
     <t>reg_03</t>
   </si>
   <si>
@@ -2666,6 +2663,9 @@
   </si>
   <si>
     <t>GA_lang</t>
+  </si>
+  <si>
+    <t>Asia Pacific</t>
   </si>
 </sst>
 </file>
@@ -3609,10 +3609,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -4979,39 +4979,39 @@
         <v>648</v>
       </c>
       <c r="B4" t="s">
-        <v>649</v>
+        <v>866</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B5" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B6" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>651</v>
+      </c>
+      <c r="B7" t="s">
         <v>652</v>
-      </c>
-      <c r="B7" t="s">
-        <v>653</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>653</v>
+      </c>
+      <c r="B8" t="s">
         <v>654</v>
-      </c>
-      <c r="B8" t="s">
-        <v>655</v>
       </c>
     </row>
   </sheetData>
@@ -5046,58 +5046,58 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>679</v>
+      </c>
+      <c r="B2" t="s">
         <v>680</v>
-      </c>
-      <c r="B2" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>681</v>
+      </c>
+      <c r="B3" t="s">
         <v>682</v>
-      </c>
-      <c r="B3" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>683</v>
+      </c>
+      <c r="B4" t="s">
         <v>684</v>
-      </c>
-      <c r="B4" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>685</v>
+      </c>
+      <c r="B5" t="s">
         <v>686</v>
-      </c>
-      <c r="B5" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>687</v>
+      </c>
+      <c r="B6" t="s">
         <v>688</v>
-      </c>
-      <c r="B6" t="s">
-        <v>689</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>689</v>
+      </c>
+      <c r="B7" t="s">
         <v>690</v>
-      </c>
-      <c r="B7" t="s">
-        <v>691</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>691</v>
+      </c>
+      <c r="B8" t="s">
         <v>692</v>
-      </c>
-      <c r="B8" t="s">
-        <v>693</v>
       </c>
     </row>
   </sheetData>
@@ -5132,18 +5132,18 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B2" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
   </sheetData>
@@ -5179,46 +5179,46 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B4" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="B5" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
   </sheetData>
@@ -5274,287 +5274,287 @@
         <v>4</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B3" t="s">
+        <v>743</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>744</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="F3" t="s">
         <v>745</v>
-      </c>
-      <c r="F3" t="s">
-        <v>746</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B4" t="s">
+        <v>746</v>
+      </c>
+      <c r="C4" t="s">
         <v>747</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
         <v>748</v>
-      </c>
-      <c r="F4" t="s">
-        <v>749</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B5" t="s">
+        <v>749</v>
+      </c>
+      <c r="C5" t="s">
         <v>750</v>
       </c>
-      <c r="C5" t="s">
-        <v>751</v>
-      </c>
       <c r="F5" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B6" t="s">
+        <v>751</v>
+      </c>
+      <c r="C6" t="s">
         <v>752</v>
       </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>753</v>
-      </c>
-      <c r="F6" t="s">
-        <v>754</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B7" t="s">
+        <v>755</v>
+      </c>
+      <c r="C7" t="s">
         <v>756</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>757</v>
-      </c>
-      <c r="F7" t="s">
-        <v>758</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B8" t="s">
+        <v>758</v>
+      </c>
+      <c r="C8" t="s">
         <v>759</v>
       </c>
-      <c r="C8" t="s">
+      <c r="F8" t="s">
         <v>760</v>
-      </c>
-      <c r="F8" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B9" t="s">
+        <v>761</v>
+      </c>
+      <c r="C9" t="s">
         <v>762</v>
       </c>
-      <c r="C9" t="s">
+      <c r="F9" t="s">
         <v>763</v>
-      </c>
-      <c r="F9" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B10" t="s">
+        <v>764</v>
+      </c>
+      <c r="C10" t="s">
+        <v>766</v>
+      </c>
+      <c r="F10" t="s">
         <v>765</v>
-      </c>
-      <c r="C10" t="s">
-        <v>767</v>
-      </c>
-      <c r="F10" t="s">
-        <v>766</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B11" t="s">
+        <v>767</v>
+      </c>
+      <c r="C11" t="s">
         <v>768</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
         <v>769</v>
-      </c>
-      <c r="F11" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B12" t="s">
+        <v>771</v>
+      </c>
+      <c r="C12" t="s">
+        <v>770</v>
+      </c>
+      <c r="F12" t="s">
         <v>772</v>
-      </c>
-      <c r="C12" t="s">
-        <v>771</v>
-      </c>
-      <c r="F12" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B13" t="s">
+        <v>773</v>
+      </c>
+      <c r="C13" t="s">
         <v>774</v>
       </c>
-      <c r="C13" t="s">
+      <c r="F13" t="s">
         <v>775</v>
-      </c>
-      <c r="F13" t="s">
-        <v>776</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="B14" t="s">
+        <v>776</v>
+      </c>
+      <c r="C14" t="s">
+        <v>778</v>
+      </c>
+      <c r="F14" t="s">
         <v>777</v>
-      </c>
-      <c r="C14" t="s">
-        <v>779</v>
-      </c>
-      <c r="F14" t="s">
-        <v>778</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B15" t="s">
+        <v>780</v>
+      </c>
+      <c r="C15" t="s">
         <v>781</v>
       </c>
-      <c r="C15" t="s">
-        <v>782</v>
-      </c>
       <c r="F15" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B16" t="s">
+        <v>782</v>
+      </c>
+      <c r="C16" t="s">
+        <v>784</v>
+      </c>
+      <c r="F16" t="s">
         <v>783</v>
-      </c>
-      <c r="C16" t="s">
-        <v>785</v>
-      </c>
-      <c r="F16" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B17" t="s">
+        <v>785</v>
+      </c>
+      <c r="C17" t="s">
         <v>786</v>
       </c>
-      <c r="C17" t="s">
+      <c r="F17" t="s">
         <v>787</v>
-      </c>
-      <c r="F17" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B18" t="s">
+        <v>788</v>
+      </c>
+      <c r="C18" t="s">
+        <v>790</v>
+      </c>
+      <c r="F18" t="s">
         <v>789</v>
-      </c>
-      <c r="C18" t="s">
-        <v>791</v>
-      </c>
-      <c r="F18" t="s">
-        <v>790</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B19" t="s">
+        <v>791</v>
+      </c>
+      <c r="C19" t="s">
         <v>792</v>
       </c>
-      <c r="C19" t="s">
+      <c r="F19" t="s">
         <v>793</v>
-      </c>
-      <c r="F19" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B20" t="s">
+        <v>794</v>
+      </c>
+      <c r="C20" t="s">
         <v>795</v>
       </c>
-      <c r="C20" t="s">
+      <c r="F20" t="s">
         <v>796</v>
-      </c>
-      <c r="F20" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="B21" t="s">
+        <v>797</v>
+      </c>
+      <c r="C21" t="s">
         <v>798</v>
       </c>
-      <c r="C21" t="s">
+      <c r="F21" t="s">
         <v>799</v>
-      </c>
-      <c r="F21" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B22" t="s">
+        <v>800</v>
+      </c>
+      <c r="C22" t="s">
         <v>801</v>
       </c>
-      <c r="C22" t="s">
+      <c r="F22" t="s">
         <v>802</v>
-      </c>
-      <c r="F22" t="s">
-        <v>803</v>
       </c>
     </row>
   </sheetData>
@@ -5608,147 +5608,147 @@
         <v>4</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B3" t="s">
+        <v>824</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>825</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="F3" s="11" t="s">
         <v>826</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>827</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B4" t="s">
+        <v>828</v>
+      </c>
+      <c r="C4" t="s">
         <v>829</v>
       </c>
-      <c r="C4" t="s">
-        <v>830</v>
-      </c>
       <c r="F4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C5" t="s">
         <v>832</v>
       </c>
-      <c r="C5" t="s">
-        <v>833</v>
-      </c>
       <c r="F5" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B6" t="s">
+        <v>834</v>
+      </c>
+      <c r="C6" t="s">
         <v>835</v>
       </c>
-      <c r="C6" t="s">
-        <v>836</v>
-      </c>
       <c r="F6" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="B7" t="s">
+        <v>836</v>
+      </c>
+      <c r="C7" t="s">
         <v>837</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>838</v>
-      </c>
-      <c r="F7" t="s">
-        <v>839</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B8" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C8" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="F8" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B9" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="C9" t="s">
+        <v>842</v>
+      </c>
+      <c r="F9" t="s">
         <v>843</v>
-      </c>
-      <c r="F9" t="s">
-        <v>844</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B10" t="s">
+        <v>845</v>
+      </c>
+      <c r="C10" t="s">
         <v>846</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
         <v>847</v>
-      </c>
-      <c r="F10" t="s">
-        <v>848</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B11" t="s">
+        <v>848</v>
+      </c>
+      <c r="C11" t="s">
         <v>849</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
         <v>850</v>
-      </c>
-      <c r="F11" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B12" t="s">
+        <v>852</v>
+      </c>
+      <c r="C12" t="s">
         <v>853</v>
       </c>
-      <c r="C12" t="s">
-        <v>854</v>
-      </c>
       <c r="F12" s="11" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
   </sheetData>
@@ -6854,10 +6854,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B3" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="C3" t="s">
         <v>479</v>
@@ -6865,21 +6865,21 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B4" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C4" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B5" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="C5" t="s">
         <v>483</v>
@@ -6887,10 +6887,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B6" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="C6" t="s">
         <v>482</v>
@@ -6898,10 +6898,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="B7" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="C7" t="s">
         <v>481</v>
@@ -6909,10 +6909,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B8" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="C8" t="s">
         <v>480</v>
@@ -6920,134 +6920,134 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B9" t="s">
+        <v>655</v>
+      </c>
+      <c r="C9" t="s">
         <v>656</v>
-      </c>
-      <c r="C9" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B10" t="s">
+        <v>661</v>
+      </c>
+      <c r="C10" t="s">
         <v>662</v>
-      </c>
-      <c r="C10" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B11" t="s">
+        <v>657</v>
+      </c>
+      <c r="C11" t="s">
         <v>658</v>
-      </c>
-      <c r="C11" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B12" t="s">
+        <v>663</v>
+      </c>
+      <c r="C12" t="s">
         <v>664</v>
-      </c>
-      <c r="C12" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B13" t="s">
+        <v>659</v>
+      </c>
+      <c r="C13" t="s">
         <v>660</v>
-      </c>
-      <c r="C13" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B14" t="s">
+        <v>667</v>
+      </c>
+      <c r="C14" t="s">
         <v>668</v>
-      </c>
-      <c r="C14" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B15" t="s">
+        <v>665</v>
+      </c>
+      <c r="C15" t="s">
         <v>666</v>
-      </c>
-      <c r="C15" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B16" t="s">
+        <v>669</v>
+      </c>
+      <c r="C16" t="s">
         <v>670</v>
-      </c>
-      <c r="C16" t="s">
-        <v>671</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B17" t="s">
+        <v>671</v>
+      </c>
+      <c r="C17" t="s">
         <v>672</v>
-      </c>
-      <c r="C17" t="s">
-        <v>673</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B18" t="s">
+        <v>675</v>
+      </c>
+      <c r="C18" t="s">
         <v>676</v>
-      </c>
-      <c r="C18" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B19" t="s">
+        <v>677</v>
+      </c>
+      <c r="C19" t="s">
         <v>678</v>
-      </c>
-      <c r="C19" t="s">
-        <v>679</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B20" t="s">
+        <v>673</v>
+      </c>
+      <c r="C20" t="s">
         <v>674</v>
-      </c>
-      <c r="C20" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -7055,21 +7055,21 @@
         <v>484</v>
       </c>
       <c r="B21" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C21" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B22" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="C22" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -7939,10 +7939,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>711</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>712</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>713</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated prj list. exresource element, list, ui added
</commit_message>
<xml_diff>
--- a/xlsx/Lists.xlsx
+++ b/xlsx/Lists.xlsx
@@ -1,33 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/o_ugur_exeter_ac_uk/Documents/Desktop/rc1.2_ou/metadata-schema/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="405" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88ED991A-AE5C-4BF0-A97E-FF7025AB0314}"/>
+  <xr:revisionPtr revIDLastSave="489" documentId="11_F25DC773A252ABDACC1048A6595D604E5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDB1C0EE-FF7D-4E2A-BA14-DDF394921354}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="18840" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="984" yWindow="1008" windowWidth="8076" windowHeight="10044" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="01_Languages" sheetId="2" r:id="rId1"/>
-    <sheet name="02_Themes" sheetId="3" r:id="rId2"/>
-    <sheet name="03_Cultural Context" sheetId="4" r:id="rId3"/>
-    <sheet name="04_Social Groups" sheetId="5" r:id="rId4"/>
-    <sheet name="05_Rights" sheetId="6" r:id="rId5"/>
-    <sheet name="06_Gender" sheetId="7" r:id="rId6"/>
-    <sheet name="07_Cultural Sensitivity" sheetId="8" r:id="rId7"/>
-    <sheet name="08_Occupations" sheetId="9" r:id="rId8"/>
-    <sheet name="09_Project Types" sheetId="10" r:id="rId9"/>
-    <sheet name="10_Project Regions" sheetId="11" r:id="rId10"/>
-    <sheet name="11_Roles" sheetId="13" r:id="rId11"/>
-    <sheet name="12_Language Labels" sheetId="15" r:id="rId12"/>
-    <sheet name="13_Authority Sources" sheetId="16" r:id="rId13"/>
-    <sheet name="14_Traditional Knowledge Labels" sheetId="17" r:id="rId14"/>
-    <sheet name="15_Biocultural Labels" sheetId="18" r:id="rId15"/>
+    <sheet name="01_Languages (OBJ,ENT)" sheetId="2" r:id="rId1"/>
+    <sheet name="02_Themes (OBJ)" sheetId="3" r:id="rId2"/>
+    <sheet name="03_Cultural Context (OBJ)" sheetId="4" r:id="rId3"/>
+    <sheet name="04_Social Groups (OBJ)" sheetId="5" r:id="rId4"/>
+    <sheet name="05_Rights (OBJ)" sheetId="6" r:id="rId5"/>
+    <sheet name="06_Gender (ENT)" sheetId="7" r:id="rId6"/>
+    <sheet name="07_Cultural Sensitivity (OBJ)" sheetId="8" r:id="rId7"/>
+    <sheet name="08_Occupations (ENT)" sheetId="9" r:id="rId8"/>
+    <sheet name="09_Project Types (COL)" sheetId="10" r:id="rId9"/>
+    <sheet name="10_Project Regions (COL)" sheetId="11" r:id="rId10"/>
+    <sheet name="11_Roles (ENT)" sheetId="13" r:id="rId11"/>
+    <sheet name="12_Language Labels (OBJ,ENT)" sheetId="15" r:id="rId12"/>
+    <sheet name="13_Authority Sources (ENT)" sheetId="16" r:id="rId13"/>
+    <sheet name="14_TraditionalKnowledge (OBJ)" sheetId="17" r:id="rId14"/>
+    <sheet name="15_Biocultural Labels (OBJ)" sheetId="18" r:id="rId15"/>
+    <sheet name="16_External Resources" sheetId="19" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="867">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="875">
   <si>
     <t>Term ID</t>
   </si>
@@ -2666,6 +2667,30 @@
   </si>
   <si>
     <t>Asia Pacific</t>
+  </si>
+  <si>
+    <t>exres_01</t>
+  </si>
+  <si>
+    <t>exres_02</t>
+  </si>
+  <si>
+    <t>exres_03</t>
+  </si>
+  <si>
+    <t>exres_04</t>
+  </si>
+  <si>
+    <t>Map</t>
+  </si>
+  <si>
+    <t>Exhibition</t>
+  </si>
+  <si>
+    <t>Channel</t>
+  </si>
+  <si>
+    <t>Interactive Form</t>
   </si>
 </sst>
 </file>
@@ -2809,10 +2834,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3078,13 +3099,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08C7DCC5-93A4-4F15-9716-2215F2C5540F}">
-  <dimension ref="A1:G140"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L140"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -3105,7 +3130,7 @@
       </c>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3126,7 +3151,7 @@
       </c>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3139,7 +3164,7 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -3152,7 +3177,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -3165,7 +3190,7 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -3178,7 +3203,7 @@
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -3191,7 +3216,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
@@ -3204,7 +3229,7 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>21</v>
       </c>
@@ -3217,7 +3242,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>23</v>
       </c>
@@ -3230,7 +3255,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>25</v>
       </c>
@@ -3243,7 +3268,7 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
@@ -3256,7 +3281,7 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>29</v>
       </c>
@@ -3267,9 +3292,8 @@
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>31</v>
       </c>
@@ -3280,9 +3304,9 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="L14" s="6"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>33</v>
       </c>
@@ -3293,9 +3317,8 @@
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>35</v>
       </c>
@@ -3305,10 +3328,8 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>37</v>
       </c>
@@ -3319,9 +3340,8 @@
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>39</v>
       </c>
@@ -3332,9 +3352,8 @@
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>41</v>
       </c>
@@ -3345,9 +3364,8 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>43</v>
       </c>
@@ -3358,9 +3376,8 @@
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>45</v>
       </c>
@@ -3371,9 +3388,8 @@
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>47</v>
       </c>
@@ -3384,9 +3400,8 @@
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>49</v>
       </c>
@@ -3399,7 +3414,7 @@
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>51</v>
       </c>
@@ -3412,7 +3427,7 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>53</v>
       </c>
@@ -3425,7 +3440,7 @@
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>55</v>
       </c>
@@ -3438,7 +3453,7 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>57</v>
       </c>
@@ -3451,7 +3466,7 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>59</v>
       </c>
@@ -3464,7 +3479,7 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>61</v>
       </c>
@@ -3477,7 +3492,7 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>63</v>
       </c>
@@ -3490,7 +3505,7 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>65</v>
       </c>
@@ -3503,7 +3518,7 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>67</v>
       </c>
@@ -3516,7 +3531,7 @@
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>69</v>
       </c>
@@ -3529,7 +3544,7 @@
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>71</v>
       </c>
@@ -3542,7 +3557,7 @@
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>73</v>
       </c>
@@ -3555,7 +3570,7 @@
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>75</v>
       </c>
@@ -3568,7 +3583,7 @@
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>76</v>
       </c>
@@ -3581,7 +3596,7 @@
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>78</v>
       </c>
@@ -3594,7 +3609,7 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>80</v>
       </c>
@@ -3607,7 +3622,7 @@
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>865</v>
       </c>
@@ -3620,7 +3635,7 @@
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>82</v>
       </c>
@@ -3633,7 +3648,7 @@
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>84</v>
       </c>
@@ -3646,7 +3661,7 @@
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>86</v>
       </c>
@@ -3659,7 +3674,7 @@
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>88</v>
       </c>
@@ -3672,7 +3687,7 @@
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>90</v>
       </c>
@@ -3685,7 +3700,7 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>92</v>
       </c>
@@ -3698,7 +3713,7 @@
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>94</v>
       </c>
@@ -3711,7 +3726,7 @@
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>96</v>
       </c>
@@ -3724,7 +3739,7 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>98</v>
       </c>
@@ -3737,7 +3752,7 @@
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>100</v>
       </c>
@@ -3750,7 +3765,7 @@
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>102</v>
       </c>
@@ -3763,7 +3778,7 @@
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>104</v>
       </c>
@@ -3776,7 +3791,7 @@
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>106</v>
       </c>
@@ -3789,7 +3804,7 @@
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>108</v>
       </c>
@@ -3802,7 +3817,7 @@
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>110</v>
       </c>
@@ -3815,7 +3830,7 @@
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>112</v>
       </c>
@@ -3828,7 +3843,7 @@
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>114</v>
       </c>
@@ -3841,7 +3856,7 @@
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>116</v>
       </c>
@@ -3854,7 +3869,7 @@
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>118</v>
       </c>
@@ -3867,7 +3882,7 @@
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>120</v>
       </c>
@@ -3880,7 +3895,7 @@
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>122</v>
       </c>
@@ -3893,7 +3908,7 @@
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>124</v>
       </c>
@@ -3906,7 +3921,7 @@
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>126</v>
       </c>
@@ -3919,7 +3934,7 @@
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>128</v>
       </c>
@@ -3932,7 +3947,7 @@
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>130</v>
       </c>
@@ -3945,7 +3960,7 @@
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>132</v>
       </c>
@@ -3958,7 +3973,7 @@
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>134</v>
       </c>
@@ -3971,7 +3986,7 @@
       <c r="F67" s="1"/>
       <c r="G67" s="1"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>136</v>
       </c>
@@ -3984,7 +3999,7 @@
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>138</v>
       </c>
@@ -3997,7 +4012,7 @@
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>140</v>
       </c>
@@ -4010,7 +4025,7 @@
       <c r="F70" s="1"/>
       <c r="G70" s="1"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>142</v>
       </c>
@@ -4023,7 +4038,7 @@
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>144</v>
       </c>
@@ -4036,7 +4051,7 @@
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>146</v>
       </c>
@@ -4049,7 +4064,7 @@
       <c r="F73" s="1"/>
       <c r="G73" s="1"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>148</v>
       </c>
@@ -4062,7 +4077,7 @@
       <c r="F74" s="1"/>
       <c r="G74" s="1"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>150</v>
       </c>
@@ -4075,7 +4090,7 @@
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>152</v>
       </c>
@@ -4088,7 +4103,7 @@
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>154</v>
       </c>
@@ -4101,7 +4116,7 @@
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>156</v>
       </c>
@@ -4114,7 +4129,7 @@
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>158</v>
       </c>
@@ -4127,7 +4142,7 @@
       <c r="F79" s="1"/>
       <c r="G79" s="1"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>160</v>
       </c>
@@ -4140,7 +4155,7 @@
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>162</v>
       </c>
@@ -4153,7 +4168,7 @@
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>164</v>
       </c>
@@ -4166,7 +4181,7 @@
       <c r="F82" s="1"/>
       <c r="G82" s="1"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>166</v>
       </c>
@@ -4179,7 +4194,7 @@
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>167</v>
       </c>
@@ -4192,7 +4207,7 @@
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>169</v>
       </c>
@@ -4205,7 +4220,7 @@
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>171</v>
       </c>
@@ -4218,7 +4233,7 @@
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>173</v>
       </c>
@@ -4231,7 +4246,7 @@
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>175</v>
       </c>
@@ -4244,7 +4259,7 @@
       <c r="F88" s="1"/>
       <c r="G88" s="1"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>177</v>
       </c>
@@ -4257,7 +4272,7 @@
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>179</v>
       </c>
@@ -4270,7 +4285,7 @@
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>181</v>
       </c>
@@ -4283,7 +4298,7 @@
       <c r="F91" s="1"/>
       <c r="G91" s="1"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>183</v>
       </c>
@@ -4296,7 +4311,7 @@
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>185</v>
       </c>
@@ -4309,7 +4324,7 @@
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>187</v>
       </c>
@@ -4322,7 +4337,7 @@
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>189</v>
       </c>
@@ -4335,7 +4350,7 @@
       <c r="F95" s="1"/>
       <c r="G95" s="1"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>191</v>
       </c>
@@ -4348,7 +4363,7 @@
       <c r="F96" s="1"/>
       <c r="G96" s="1"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>193</v>
       </c>
@@ -4361,7 +4376,7 @@
       <c r="F97" s="1"/>
       <c r="G97" s="1"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>195</v>
       </c>
@@ -4374,7 +4389,7 @@
       <c r="F98" s="1"/>
       <c r="G98" s="1"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>197</v>
       </c>
@@ -4387,7 +4402,7 @@
       <c r="F99" s="1"/>
       <c r="G99" s="1"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>199</v>
       </c>
@@ -4400,7 +4415,7 @@
       <c r="F100" s="1"/>
       <c r="G100" s="1"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>201</v>
       </c>
@@ -4413,7 +4428,7 @@
       <c r="F101" s="1"/>
       <c r="G101" s="1"/>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>203</v>
       </c>
@@ -4426,7 +4441,7 @@
       <c r="F102" s="1"/>
       <c r="G102" s="1"/>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>205</v>
       </c>
@@ -4439,7 +4454,7 @@
       <c r="F103" s="1"/>
       <c r="G103" s="1"/>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>207</v>
       </c>
@@ -4452,7 +4467,7 @@
       <c r="F104" s="1"/>
       <c r="G104" s="1"/>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>209</v>
       </c>
@@ -4465,7 +4480,7 @@
       <c r="F105" s="1"/>
       <c r="G105" s="1"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>211</v>
       </c>
@@ -4478,7 +4493,7 @@
       <c r="F106" s="1"/>
       <c r="G106" s="1"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>213</v>
       </c>
@@ -4491,7 +4506,7 @@
       <c r="F107" s="1"/>
       <c r="G107" s="1"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>215</v>
       </c>
@@ -4504,7 +4519,7 @@
       <c r="F108" s="1"/>
       <c r="G108" s="1"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>217</v>
       </c>
@@ -4517,7 +4532,7 @@
       <c r="F109" s="1"/>
       <c r="G109" s="1"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>219</v>
       </c>
@@ -4530,7 +4545,7 @@
       <c r="F110" s="1"/>
       <c r="G110" s="1"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>221</v>
       </c>
@@ -4543,7 +4558,7 @@
       <c r="F111" s="1"/>
       <c r="G111" s="1"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>223</v>
       </c>
@@ -4556,7 +4571,7 @@
       <c r="F112" s="1"/>
       <c r="G112" s="1"/>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>225</v>
       </c>
@@ -4569,7 +4584,7 @@
       <c r="F113" s="1"/>
       <c r="G113" s="1"/>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>227</v>
       </c>
@@ -4582,7 +4597,7 @@
       <c r="F114" s="1"/>
       <c r="G114" s="1"/>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>229</v>
       </c>
@@ -4595,7 +4610,7 @@
       <c r="F115" s="1"/>
       <c r="G115" s="1"/>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>231</v>
       </c>
@@ -4608,7 +4623,7 @@
       <c r="F116" s="1"/>
       <c r="G116" s="1"/>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>233</v>
       </c>
@@ -4621,7 +4636,7 @@
       <c r="F117" s="1"/>
       <c r="G117" s="1"/>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>235</v>
       </c>
@@ -4634,7 +4649,7 @@
       <c r="F118" s="1"/>
       <c r="G118" s="1"/>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>237</v>
       </c>
@@ -4647,7 +4662,7 @@
       <c r="F119" s="1"/>
       <c r="G119" s="1"/>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>239</v>
       </c>
@@ -4660,7 +4675,7 @@
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>241</v>
       </c>
@@ -4673,7 +4688,7 @@
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>243</v>
       </c>
@@ -4686,7 +4701,7 @@
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>245</v>
       </c>
@@ -4699,7 +4714,7 @@
       <c r="F123" s="1"/>
       <c r="G123" s="1"/>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>247</v>
       </c>
@@ -4712,7 +4727,7 @@
       <c r="F124" s="1"/>
       <c r="G124" s="1"/>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>248</v>
       </c>
@@ -4725,7 +4740,7 @@
       <c r="F125" s="1"/>
       <c r="G125" s="1"/>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>250</v>
       </c>
@@ -4738,7 +4753,7 @@
       <c r="F126" s="1"/>
       <c r="G126" s="1"/>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>252</v>
       </c>
@@ -4751,7 +4766,7 @@
       <c r="F127" s="1"/>
       <c r="G127" s="1"/>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>254</v>
       </c>
@@ -4764,7 +4779,7 @@
       <c r="F128" s="1"/>
       <c r="G128" s="1"/>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>256</v>
       </c>
@@ -4777,7 +4792,7 @@
       <c r="F129" s="1"/>
       <c r="G129" s="1"/>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>258</v>
       </c>
@@ -4790,7 +4805,7 @@
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>260</v>
       </c>
@@ -4803,7 +4818,7 @@
       <c r="F131" s="1"/>
       <c r="G131" s="1"/>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>262</v>
       </c>
@@ -4816,7 +4831,7 @@
       <c r="F132" s="1"/>
       <c r="G132" s="1"/>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>264</v>
       </c>
@@ -4829,7 +4844,7 @@
       <c r="F133" s="1"/>
       <c r="G133" s="1"/>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>266</v>
       </c>
@@ -4842,7 +4857,7 @@
       <c r="F134" s="1"/>
       <c r="G134" s="1"/>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>268</v>
       </c>
@@ -4855,7 +4870,7 @@
       <c r="F135" s="1"/>
       <c r="G135" s="1"/>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>270</v>
       </c>
@@ -4868,7 +4883,7 @@
       <c r="F136" s="1"/>
       <c r="G136" s="1"/>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>272</v>
       </c>
@@ -4881,7 +4896,7 @@
       <c r="F137" s="1"/>
       <c r="G137" s="1"/>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>274</v>
       </c>
@@ -4894,7 +4909,7 @@
       <c r="F138" s="1"/>
       <c r="G138" s="1"/>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>276</v>
       </c>
@@ -4907,7 +4922,7 @@
       <c r="F139" s="1"/>
       <c r="G139" s="1"/>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -4924,9 +4939,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{539D0DAF-3B47-4A29-A75D-3D6ADB320449}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -4946,7 +4961,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4966,7 +4981,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>646</v>
       </c>
@@ -4974,7 +4989,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>648</v>
       </c>
@@ -4982,7 +4997,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>649</v>
       </c>
@@ -4990,7 +5005,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>650</v>
       </c>
@@ -4998,7 +5013,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>651</v>
       </c>
@@ -5006,7 +5021,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>653</v>
       </c>
@@ -5022,9 +5037,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F350B9F1-06F7-4E8A-B44A-16E139FB0B1D}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5044,7 +5059,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>679</v>
       </c>
@@ -5052,7 +5067,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>681</v>
       </c>
@@ -5060,7 +5075,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>683</v>
       </c>
@@ -5068,7 +5083,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>685</v>
       </c>
@@ -5076,7 +5091,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>687</v>
       </c>
@@ -5084,7 +5099,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>689</v>
       </c>
@@ -5092,7 +5107,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>691</v>
       </c>
@@ -5108,9 +5123,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5D6CC2-7C88-44F7-8C63-8AD47A42CD2B}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5130,7 +5145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>695</v>
       </c>
@@ -5138,7 +5153,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>696</v>
       </c>
@@ -5155,9 +5170,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9990D756-E521-44BC-87A8-D4E80EBBCAC7}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5177,7 +5192,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>699</v>
       </c>
@@ -5188,7 +5203,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>700</v>
       </c>
@@ -5199,7 +5214,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>701</v>
       </c>
@@ -5210,7 +5225,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>702</v>
       </c>
@@ -5230,14 +5245,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13F67E00-EC1B-4E47-80B8-6C2ADC61550B}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -5257,7 +5272,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -5277,7 +5292,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>804</v>
       </c>
@@ -5291,7 +5306,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>805</v>
       </c>
@@ -5305,7 +5320,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>806</v>
       </c>
@@ -5319,7 +5334,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>807</v>
       </c>
@@ -5333,7 +5348,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>808</v>
       </c>
@@ -5347,7 +5362,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>809</v>
       </c>
@@ -5361,7 +5376,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>810</v>
       </c>
@@ -5375,7 +5390,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>811</v>
       </c>
@@ -5389,7 +5404,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>812</v>
       </c>
@@ -5403,7 +5418,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>813</v>
       </c>
@@ -5417,7 +5432,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>814</v>
       </c>
@@ -5431,7 +5446,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>815</v>
       </c>
@@ -5445,7 +5460,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>816</v>
       </c>
@@ -5459,7 +5474,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>817</v>
       </c>
@@ -5473,7 +5488,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>818</v>
       </c>
@@ -5487,7 +5502,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>819</v>
       </c>
@@ -5501,7 +5516,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>820</v>
       </c>
@@ -5515,7 +5530,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>821</v>
       </c>
@@ -5529,7 +5544,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>822</v>
       </c>
@@ -5543,7 +5558,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>823</v>
       </c>
@@ -5565,13 +5580,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F3B1DC4-7228-4E7B-AE10-2426AE58FF55}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -5591,7 +5606,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -5611,7 +5626,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>854</v>
       </c>
@@ -5625,7 +5640,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>855</v>
       </c>
@@ -5639,7 +5654,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>856</v>
       </c>
@@ -5653,7 +5668,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>857</v>
       </c>
@@ -5667,7 +5682,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>858</v>
       </c>
@@ -5681,7 +5696,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>859</v>
       </c>
@@ -5695,7 +5710,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>860</v>
       </c>
@@ -5709,7 +5724,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>861</v>
       </c>
@@ -5723,7 +5738,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>862</v>
       </c>
@@ -5737,7 +5752,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>863</v>
       </c>
@@ -5760,16 +5775,104 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A254189-A980-43BE-BE8F-0FFFAFD05AA6}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>867</v>
+      </c>
+      <c r="B3" t="s">
+        <v>871</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="F3" s="11"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>868</v>
+      </c>
+      <c r="B4" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>869</v>
+      </c>
+      <c r="B5" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>870</v>
+      </c>
+      <c r="B6" t="s">
+        <v>874</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{477AB8E0-193B-4ACE-9281-1EB5DE711D3C}">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -5789,7 +5892,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -5809,7 +5912,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>278</v>
       </c>
@@ -5820,7 +5923,7 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>280</v>
       </c>
@@ -5831,7 +5934,7 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>282</v>
       </c>
@@ -5842,7 +5945,7 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>284</v>
       </c>
@@ -5853,7 +5956,7 @@
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>286</v>
       </c>
@@ -5864,7 +5967,7 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>288</v>
       </c>
@@ -5875,7 +5978,7 @@
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>290</v>
       </c>
@@ -5895,7 +5998,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>295</v>
       </c>
@@ -5906,7 +6009,7 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>297</v>
       </c>
@@ -5917,7 +6020,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>299</v>
       </c>
@@ -5928,7 +6031,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>301</v>
       </c>
@@ -5939,7 +6042,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>303</v>
       </c>
@@ -5950,7 +6053,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>305</v>
       </c>
@@ -5961,7 +6064,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>307</v>
       </c>
@@ -5972,7 +6075,7 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>309</v>
       </c>
@@ -5983,7 +6086,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>311</v>
       </c>
@@ -5994,7 +6097,7 @@
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>313</v>
       </c>
@@ -6005,7 +6108,7 @@
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>315</v>
       </c>
@@ -6016,7 +6119,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>317</v>
       </c>
@@ -6027,7 +6130,7 @@
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>319</v>
       </c>
@@ -6038,7 +6141,7 @@
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>321</v>
       </c>
@@ -6049,7 +6152,7 @@
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>323</v>
       </c>
@@ -6060,7 +6163,7 @@
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>325</v>
       </c>
@@ -6071,7 +6174,7 @@
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>327</v>
       </c>
@@ -6082,7 +6185,7 @@
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>329</v>
       </c>
@@ -6093,7 +6196,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>331</v>
       </c>
@@ -6101,7 +6204,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>333</v>
       </c>
@@ -6109,7 +6212,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>335</v>
       </c>
@@ -6117,7 +6220,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>337</v>
       </c>
@@ -6125,7 +6228,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>339</v>
       </c>
@@ -6141,16 +6244,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E16B73E5-B011-40A2-8AFF-3FBA72B05675}">
   <dimension ref="A1:F33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="32.42578125" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="32.44140625" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -6170,7 +6273,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -6190,7 +6293,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>341</v>
       </c>
@@ -6199,7 +6302,7 @@
       </c>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>343</v>
       </c>
@@ -6207,7 +6310,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>345</v>
       </c>
@@ -6215,7 +6318,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>347</v>
       </c>
@@ -6223,7 +6326,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>349</v>
       </c>
@@ -6231,7 +6334,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>351</v>
       </c>
@@ -6239,7 +6342,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>353</v>
       </c>
@@ -6247,7 +6350,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>355</v>
       </c>
@@ -6255,7 +6358,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>357</v>
       </c>
@@ -6263,7 +6366,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>359</v>
       </c>
@@ -6271,7 +6374,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>361</v>
       </c>
@@ -6279,7 +6382,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>363</v>
       </c>
@@ -6287,7 +6390,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>365</v>
       </c>
@@ -6295,7 +6398,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>367</v>
       </c>
@@ -6303,7 +6406,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>369</v>
       </c>
@@ -6311,7 +6414,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>371</v>
       </c>
@@ -6319,7 +6422,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>373</v>
       </c>
@@ -6327,7 +6430,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>375</v>
       </c>
@@ -6335,7 +6438,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>377</v>
       </c>
@@ -6343,7 +6446,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>379</v>
       </c>
@@ -6351,7 +6454,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>381</v>
       </c>
@@ -6359,7 +6462,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>383</v>
       </c>
@@ -6367,7 +6470,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>385</v>
       </c>
@@ -6375,7 +6478,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>387</v>
       </c>
@@ -6383,7 +6486,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>389</v>
       </c>
@@ -6391,7 +6494,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>391</v>
       </c>
@@ -6399,7 +6502,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>393</v>
       </c>
@@ -6407,7 +6510,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>395</v>
       </c>
@@ -6415,7 +6518,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>397</v>
       </c>
@@ -6423,7 +6526,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>399</v>
       </c>
@@ -6431,7 +6534,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>401</v>
       </c>
@@ -6447,13 +6550,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3BBE258-A0AD-4181-B80C-BA0C0B18114A}">
   <dimension ref="A1:F40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -6473,7 +6576,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -6493,7 +6596,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>403</v>
       </c>
@@ -6501,7 +6604,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>405</v>
       </c>
@@ -6509,7 +6612,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>407</v>
       </c>
@@ -6517,7 +6620,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>409</v>
       </c>
@@ -6525,7 +6628,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>411</v>
       </c>
@@ -6533,7 +6636,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>413</v>
       </c>
@@ -6541,7 +6644,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>415</v>
       </c>
@@ -6549,7 +6652,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>417</v>
       </c>
@@ -6557,7 +6660,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>419</v>
       </c>
@@ -6565,7 +6668,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>421</v>
       </c>
@@ -6573,7 +6676,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>423</v>
       </c>
@@ -6581,7 +6684,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>425</v>
       </c>
@@ -6589,7 +6692,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>427</v>
       </c>
@@ -6597,7 +6700,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>429</v>
       </c>
@@ -6605,7 +6708,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>431</v>
       </c>
@@ -6613,7 +6716,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>433</v>
       </c>
@@ -6621,7 +6724,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>435</v>
       </c>
@@ -6629,7 +6732,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>437</v>
       </c>
@@ -6637,7 +6740,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>439</v>
       </c>
@@ -6645,7 +6748,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>441</v>
       </c>
@@ -6653,7 +6756,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>443</v>
       </c>
@@ -6661,7 +6764,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>445</v>
       </c>
@@ -6669,7 +6772,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>447</v>
       </c>
@@ -6677,7 +6780,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>449</v>
       </c>
@@ -6685,7 +6788,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>451</v>
       </c>
@@ -6693,7 +6796,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>453</v>
       </c>
@@ -6701,7 +6804,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>455</v>
       </c>
@@ -6709,7 +6812,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>457</v>
       </c>
@@ -6717,7 +6820,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>459</v>
       </c>
@@ -6725,7 +6828,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>461</v>
       </c>
@@ -6733,7 +6836,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>463</v>
       </c>
@@ -6741,7 +6844,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>465</v>
       </c>
@@ -6749,7 +6852,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>467</v>
       </c>
@@ -6757,7 +6860,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>469</v>
       </c>
@@ -6765,7 +6868,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>471</v>
       </c>
@@ -6773,7 +6876,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>473</v>
       </c>
@@ -6781,7 +6884,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>475</v>
       </c>
@@ -6789,7 +6892,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>477</v>
       </c>
@@ -6805,14 +6908,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B29326D-C093-4910-A1C0-5F486B1575C8}">
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="2" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="100.85546875" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="59.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="100.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -6832,7 +6935,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -6852,7 +6955,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>721</v>
       </c>
@@ -6863,7 +6966,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>722</v>
       </c>
@@ -6874,7 +6977,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>740</v>
       </c>
@@ -6885,7 +6988,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>723</v>
       </c>
@@ -6896,7 +6999,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>724</v>
       </c>
@@ -6907,7 +7010,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>725</v>
       </c>
@@ -6918,7 +7021,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>726</v>
       </c>
@@ -6929,7 +7032,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>727</v>
       </c>
@@ -6940,7 +7043,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>728</v>
       </c>
@@ -6951,7 +7054,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>729</v>
       </c>
@@ -6962,7 +7065,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>730</v>
       </c>
@@ -6973,7 +7076,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>731</v>
       </c>
@@ -6984,7 +7087,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>732</v>
       </c>
@@ -6995,7 +7098,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>733</v>
       </c>
@@ -7006,7 +7109,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>734</v>
       </c>
@@ -7017,7 +7120,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>735</v>
       </c>
@@ -7028,7 +7131,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>736</v>
       </c>
@@ -7039,7 +7142,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>737</v>
       </c>
@@ -7050,7 +7153,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>484</v>
       </c>
@@ -7061,7 +7164,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>738</v>
       </c>
@@ -7072,16 +7175,16 @@
         <v>742</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C23" s="9"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C24" s="9"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C25" s="9"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C26" s="9"/>
     </row>
   </sheetData>
@@ -7092,9 +7195,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB7B9CC8-1CF9-4C25-9399-8780B24CD111}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>1</v>
       </c>
@@ -7114,7 +7217,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -7134,7 +7237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>485</v>
       </c>
@@ -7142,7 +7245,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>487</v>
       </c>
@@ -7150,7 +7253,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>489</v>
       </c>
@@ -7159,7 +7262,7 @@
       </c>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>491</v>
       </c>
@@ -7175,12 +7278,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54A83176-2C03-4098-BDEE-3DBB9068115F}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>1</v>
       </c>
@@ -7200,7 +7303,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -7220,7 +7323,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>493</v>
       </c>
@@ -7231,7 +7334,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>496</v>
       </c>
@@ -7242,7 +7345,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>499</v>
       </c>
@@ -7261,13 +7364,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA4C0B3A-7FCD-4BED-A793-C85D90A184F8}">
   <dimension ref="A1:J69"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="23.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -7287,7 +7390,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -7310,7 +7413,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>503</v>
       </c>
@@ -7318,7 +7421,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>505</v>
       </c>
@@ -7326,7 +7429,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>507</v>
       </c>
@@ -7334,7 +7437,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>509</v>
       </c>
@@ -7342,7 +7445,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>511</v>
       </c>
@@ -7350,7 +7453,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>513</v>
       </c>
@@ -7358,7 +7461,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>515</v>
       </c>
@@ -7366,7 +7469,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>517</v>
       </c>
@@ -7374,7 +7477,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>519</v>
       </c>
@@ -7382,7 +7485,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>521</v>
       </c>
@@ -7390,7 +7493,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>523</v>
       </c>
@@ -7398,7 +7501,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>525</v>
       </c>
@@ -7406,7 +7509,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>527</v>
       </c>
@@ -7414,7 +7517,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>529</v>
       </c>
@@ -7422,7 +7525,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>531</v>
       </c>
@@ -7430,7 +7533,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>533</v>
       </c>
@@ -7438,7 +7541,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>535</v>
       </c>
@@ -7446,7 +7549,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>537</v>
       </c>
@@ -7454,7 +7557,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>539</v>
       </c>
@@ -7462,7 +7565,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>541</v>
       </c>
@@ -7470,7 +7573,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>543</v>
       </c>
@@ -7478,7 +7581,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>545</v>
       </c>
@@ -7486,7 +7589,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>547</v>
       </c>
@@ -7494,7 +7597,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>549</v>
       </c>
@@ -7502,7 +7605,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>551</v>
       </c>
@@ -7510,7 +7613,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>553</v>
       </c>
@@ -7518,7 +7621,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>555</v>
       </c>
@@ -7526,7 +7629,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>557</v>
       </c>
@@ -7534,7 +7637,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>559</v>
       </c>
@@ -7542,7 +7645,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>561</v>
       </c>
@@ -7550,7 +7653,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>563</v>
       </c>
@@ -7558,7 +7661,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>565</v>
       </c>
@@ -7566,7 +7669,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>567</v>
       </c>
@@ -7574,7 +7677,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>569</v>
       </c>
@@ -7582,7 +7685,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>571</v>
       </c>
@@ -7590,7 +7693,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>573</v>
       </c>
@@ -7598,7 +7701,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>575</v>
       </c>
@@ -7606,7 +7709,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>577</v>
       </c>
@@ -7614,7 +7717,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>579</v>
       </c>
@@ -7622,7 +7725,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>581</v>
       </c>
@@ -7630,7 +7733,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>583</v>
       </c>
@@ -7638,7 +7741,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>585</v>
       </c>
@@ -7646,7 +7749,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>587</v>
       </c>
@@ -7654,7 +7757,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>589</v>
       </c>
@@ -7662,7 +7765,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>591</v>
       </c>
@@ -7670,7 +7773,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>593</v>
       </c>
@@ -7678,7 +7781,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>595</v>
       </c>
@@ -7686,7 +7789,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>597</v>
       </c>
@@ -7694,7 +7797,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>599</v>
       </c>
@@ -7702,7 +7805,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>601</v>
       </c>
@@ -7710,7 +7813,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>603</v>
       </c>
@@ -7718,7 +7821,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>605</v>
       </c>
@@ -7726,7 +7829,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>607</v>
       </c>
@@ -7734,7 +7837,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>609</v>
       </c>
@@ -7742,7 +7845,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>611</v>
       </c>
@@ -7750,7 +7853,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>613</v>
       </c>
@@ -7758,7 +7861,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>615</v>
       </c>
@@ -7766,7 +7869,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>617</v>
       </c>
@@ -7774,7 +7877,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>619</v>
       </c>
@@ -7782,7 +7885,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>621</v>
       </c>
@@ -7790,7 +7893,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>623</v>
       </c>
@@ -7798,7 +7901,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>625</v>
       </c>
@@ -7806,7 +7909,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>627</v>
       </c>
@@ -7814,7 +7917,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>629</v>
       </c>
@@ -7822,7 +7925,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>631</v>
       </c>
@@ -7830,7 +7933,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>633</v>
       </c>
@@ -7841,7 +7944,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>636</v>
       </c>
@@ -7860,12 +7963,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F08A626F-F860-4615-8CDE-0A8AB0EDDB54}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -7885,7 +7988,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -7905,7 +8008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>638</v>
       </c>
@@ -7913,7 +8016,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>640</v>
       </c>
@@ -7921,7 +8024,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>642</v>
       </c>
@@ -7929,7 +8032,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>644</v>
       </c>
@@ -7937,7 +8040,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>711</v>
       </c>

</xml_diff>